<commit_message>
feat: JobPosting page and candidates excel downloading feature added
</commit_message>
<xml_diff>
--- a/backend/data/67b48d4517400d87f1df4610.xlsx
+++ b/backend/data/67b48d4517400d87f1df4610.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -465,9 +465,20 @@
         <v>115</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v xml:space="preserve">Dhanush </v>
+      </c>
+      <c r="B7" t="str">
+        <v>dhanush4300@gmail.com</v>
+      </c>
+      <c r="C7">
+        <v>65</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>